<commit_message>
Realizacion de estados de conformidades
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO ODC.xlsx
+++ b/storage/app/templates/FORMATO ODC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adv\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910A5809-7F2B-401C-A507-559BB161408D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E21DC67-161A-4D6C-A076-BA66186F845E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="1" xr2:uid="{CD2C727A-B478-40DC-A0A5-37EBD1630B47}"/>
   </bookViews>
@@ -603,7 +603,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -624,68 +624,17 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
@@ -693,56 +642,11 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -755,18 +659,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
@@ -776,6 +668,152 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -785,6 +823,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -809,33 +850,38 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -846,70 +892,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares 3" xfId="2" xr:uid="{60AA6EFA-E802-43AC-A264-3B3C3439C925}"/>
@@ -1315,50 +1316,50 @@
   </cols>
   <sheetData>
     <row r="6" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="66"/>
-      <c r="C6" s="77" t="s">
+      <c r="B6" s="80"/>
+      <c r="C6" s="83" t="s">
         <v>48</v>
       </c>
-      <c r="D6" s="69"/>
-      <c r="E6" s="69"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="35" t="s">
+      <c r="D6" s="84"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="36"/>
+      <c r="H6" s="42"/>
     </row>
     <row r="7" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="67"/>
-      <c r="C7" s="71"/>
-      <c r="D7" s="72"/>
-      <c r="E7" s="72"/>
-      <c r="F7" s="73"/>
-      <c r="G7" s="35" t="s">
+      <c r="B7" s="81"/>
+      <c r="C7" s="86"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="88"/>
+      <c r="G7" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="36"/>
+      <c r="H7" s="42"/>
     </row>
     <row r="8" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="67"/>
-      <c r="C8" s="71"/>
-      <c r="D8" s="72"/>
-      <c r="E8" s="72"/>
-      <c r="F8" s="73"/>
-      <c r="G8" s="35" t="s">
+      <c r="B8" s="81"/>
+      <c r="C8" s="86"/>
+      <c r="D8" s="87"/>
+      <c r="E8" s="87"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="36"/>
+      <c r="H8" s="42"/>
     </row>
     <row r="9" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="68"/>
-      <c r="C9" s="74"/>
-      <c r="D9" s="75"/>
-      <c r="E9" s="75"/>
-      <c r="F9" s="76"/>
-      <c r="G9" s="35" t="s">
+      <c r="B9" s="82"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="90"/>
+      <c r="F9" s="91"/>
+      <c r="G9" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="H9" s="36"/>
+      <c r="H9" s="42"/>
     </row>
     <row r="10" spans="2:8" ht="21" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
@@ -1370,179 +1371,179 @@
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="2:8" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="83" t="s">
+      <c r="B11" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="84"/>
-      <c r="D11" s="48"/>
-      <c r="E11" s="49"/>
-      <c r="F11" s="49"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="51"/>
+      <c r="C11" s="50"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="19"/>
     </row>
     <row r="12" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="85" t="s">
+      <c r="B12" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="78"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="55" t="s">
+      <c r="C12" s="52"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="56"/>
+      <c r="H12" s="54"/>
     </row>
     <row r="13" spans="2:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="86" t="s">
+      <c r="B13" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="79"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="53"/>
-      <c r="F13" s="53"/>
-      <c r="G13" s="55" t="s">
+      <c r="C13" s="30"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="H13" s="56"/>
+      <c r="H13" s="54"/>
     </row>
     <row r="14" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="85" t="s">
+      <c r="B14" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="78"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="53"/>
-      <c r="F14" s="53"/>
-      <c r="G14" s="62"/>
-      <c r="H14" s="64"/>
+      <c r="C14" s="52"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="28"/>
     </row>
     <row r="15" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B15" s="57"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="65"/>
-      <c r="E15" s="59"/>
-      <c r="F15" s="59"/>
-      <c r="G15" s="60"/>
-      <c r="H15" s="61"/>
+      <c r="B15" s="55"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="25"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B16" s="82"/>
+      <c r="B16" s="31"/>
     </row>
     <row r="17" spans="2:8" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="97" t="s">
+      <c r="B17" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="23"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="43"/>
+      <c r="G17" s="43"/>
+      <c r="H17" s="44"/>
     </row>
     <row r="18" spans="2:8" ht="6.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="103"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="25"/>
+      <c r="B18" s="36"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="11"/>
     </row>
     <row r="19" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="41"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="42" t="s">
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="26"/>
+      <c r="H19" s="46"/>
     </row>
     <row r="20" spans="2:8" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="103"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="41"/>
-      <c r="G20" s="41"/>
-      <c r="H20" s="25"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="11"/>
     </row>
     <row r="21" spans="2:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="44" t="s">
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="28"/>
+      <c r="H21" s="58"/>
     </row>
     <row r="22" spans="2:8" ht="12.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="29"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="30"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="13"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="32"/>
+      <c r="C23" s="60"/>
+      <c r="D23" s="60"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="61"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B24" s="29"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="30"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="13"/>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="46"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="30"/>
+      <c r="C25" s="60"/>
+      <c r="D25" s="60"/>
+      <c r="E25" s="60"/>
+      <c r="F25" s="60"/>
+      <c r="G25" s="60"/>
+      <c r="H25" s="13"/>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B26" s="29"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="30"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="13"/>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B27" s="33" t="s">
+      <c r="B27" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="34"/>
+      <c r="C27" s="69"/>
+      <c r="D27" s="69"/>
+      <c r="E27" s="69"/>
+      <c r="F27" s="69"/>
+      <c r="G27" s="69"/>
+      <c r="H27" s="70"/>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B28" s="5"/>
@@ -1554,503 +1555,511 @@
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B29" s="82"/>
-      <c r="C29" s="82"/>
-      <c r="D29" s="82"/>
-      <c r="E29" s="82"/>
-      <c r="F29" s="82"/>
-      <c r="G29" s="82"/>
-      <c r="H29" s="82"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
     </row>
     <row r="30" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B30" s="98" t="s">
+      <c r="B30" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="D30" s="10"/>
-      <c r="E30" s="11" t="s">
+      <c r="D30" s="66"/>
+      <c r="E30" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="F30" s="11" t="s">
+      <c r="F30" s="67" t="s">
         <v>3</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H30" s="100" t="s">
+      <c r="H30" s="34" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="31" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B31" s="99"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
+      <c r="B31" s="64"/>
+      <c r="C31" s="65"/>
+      <c r="D31" s="66"/>
+      <c r="E31" s="67"/>
+      <c r="F31" s="67"/>
       <c r="G31" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H31" s="101" t="s">
+      <c r="H31" s="35" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="2:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="38" t="s">
+      <c r="B32" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="39" t="s">
+      <c r="C32" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="39"/>
-      <c r="E32" s="38" t="s">
+      <c r="D32" s="62"/>
+      <c r="E32" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F32" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="F32" s="38" t="s">
+      <c r="G32" s="111" t="s">
+        <v>46</v>
+      </c>
+      <c r="H32" s="111" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" ht="19.8" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" s="62" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="62"/>
+      <c r="E33" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="G32" s="40" t="s">
+      <c r="F33" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="G33" s="111" t="s">
         <v>46</v>
       </c>
-      <c r="H32" s="40" t="s">
+      <c r="H33" s="111" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="2:8" ht="19.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="38" t="s">
+    <row r="34" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C33" s="39" t="s">
+      <c r="C34" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="D33" s="39"/>
-      <c r="E33" s="38" t="s">
+      <c r="D34" s="62"/>
+      <c r="E34" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F34" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="F33" s="38" t="s">
+      <c r="G34" s="111" t="s">
+        <v>46</v>
+      </c>
+      <c r="H34" s="111" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" ht="16.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B35" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C35" s="62" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="62"/>
+      <c r="E35" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="G33" s="40" t="s">
+      <c r="F35" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="G35" s="111" t="s">
         <v>46</v>
       </c>
-      <c r="H33" s="40" t="s">
+      <c r="H35" s="111" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="38" t="s">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B36" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="39" t="s">
+      <c r="C36" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="D34" s="39"/>
-      <c r="E34" s="38" t="s">
+      <c r="D36" s="62"/>
+      <c r="E36" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F36" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="F34" s="38" t="s">
+      <c r="G36" s="111" t="s">
+        <v>46</v>
+      </c>
+      <c r="H36" s="111" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B37" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" s="62" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37" s="62"/>
+      <c r="E37" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="G34" s="40" t="s">
+      <c r="F37" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="G37" s="111" t="s">
         <v>46</v>
       </c>
-      <c r="H34" s="40" t="s">
+      <c r="H37" s="111" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="2:8" ht="16.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="38" t="s">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B38" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="39" t="s">
+      <c r="C38" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="D35" s="39"/>
-      <c r="E35" s="38" t="s">
+      <c r="D38" s="62"/>
+      <c r="E38" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F38" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="F35" s="38" t="s">
+      <c r="G38" s="111" t="s">
+        <v>46</v>
+      </c>
+      <c r="H38" s="111" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B39" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39" s="62" t="s">
+        <v>40</v>
+      </c>
+      <c r="D39" s="62"/>
+      <c r="E39" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="G35" s="40" t="s">
+      <c r="F39" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="G39" s="111" t="s">
         <v>46</v>
       </c>
-      <c r="H35" s="40" t="s">
+      <c r="H39" s="111" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B36" s="38" t="s">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B40" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="39" t="s">
+      <c r="C40" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="39"/>
-      <c r="E36" s="38" t="s">
+      <c r="D40" s="62"/>
+      <c r="E40" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F40" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="F36" s="38" t="s">
+      <c r="G40" s="111" t="s">
+        <v>46</v>
+      </c>
+      <c r="H40" s="111" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B41" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C41" s="62" t="s">
+        <v>40</v>
+      </c>
+      <c r="D41" s="62"/>
+      <c r="E41" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="G36" s="40" t="s">
+      <c r="F41" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="G41" s="111" t="s">
         <v>46</v>
       </c>
-      <c r="H36" s="40" t="s">
+      <c r="H41" s="111" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B37" s="38" t="s">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B42" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C37" s="39" t="s">
+      <c r="C42" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="D37" s="39"/>
-      <c r="E37" s="38" t="s">
+      <c r="D42" s="62"/>
+      <c r="E42" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F42" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="F37" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="G37" s="40" t="s">
+      <c r="G42" s="111" t="s">
         <v>46</v>
       </c>
-      <c r="H37" s="40" t="s">
+      <c r="H42" s="111" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B38" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="D38" s="39"/>
-      <c r="E38" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="F38" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="G38" s="40" t="s">
-        <v>46</v>
-      </c>
-      <c r="H38" s="40" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B39" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="C39" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="D39" s="39"/>
-      <c r="E39" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="F39" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="G39" s="40" t="s">
-        <v>46</v>
-      </c>
-      <c r="H39" s="40" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B40" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="C40" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="D40" s="39"/>
-      <c r="E40" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="F40" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="G40" s="40" t="s">
-        <v>46</v>
-      </c>
-      <c r="H40" s="40" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B41" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="C41" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="D41" s="39"/>
-      <c r="E41" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="F41" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="G41" s="40" t="s">
-        <v>46</v>
-      </c>
-      <c r="H41" s="40" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B42" s="38" t="s">
-        <v>39</v>
-      </c>
-      <c r="C42" s="39" t="s">
-        <v>40</v>
-      </c>
-      <c r="D42" s="39"/>
-      <c r="E42" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="F42" s="38" t="s">
-        <v>42</v>
-      </c>
-      <c r="G42" s="40" t="s">
-        <v>46</v>
-      </c>
-      <c r="H42" s="40" t="s">
-        <v>47</v>
-      </c>
-    </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-      <c r="F43" s="12"/>
-      <c r="G43" s="12"/>
-      <c r="H43" s="12"/>
+      <c r="B43" s="98"/>
+      <c r="C43" s="98"/>
+      <c r="D43" s="98"/>
+      <c r="E43" s="98"/>
+      <c r="F43" s="98"/>
+      <c r="G43" s="98"/>
+      <c r="H43" s="98"/>
     </row>
     <row r="44" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B44" s="13"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="15" t="s">
+      <c r="B44" s="99"/>
+      <c r="C44" s="100"/>
+      <c r="D44" s="100"/>
+      <c r="E44" s="100"/>
+      <c r="F44" s="101" t="s">
         <v>20</v>
       </c>
-      <c r="G44" s="16"/>
-      <c r="H44" s="17"/>
+      <c r="G44" s="102"/>
+      <c r="H44" s="8"/>
     </row>
     <row r="45" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B45" s="15" t="s">
+      <c r="B45" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="C45" s="16"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
-      <c r="F45" s="15" t="s">
+      <c r="C45" s="102"/>
+      <c r="D45" s="102"/>
+      <c r="E45" s="102"/>
+      <c r="F45" s="101" t="s">
         <v>21</v>
       </c>
-      <c r="G45" s="16"/>
-      <c r="H45" s="17"/>
+      <c r="G45" s="102"/>
+      <c r="H45" s="8"/>
     </row>
     <row r="46" spans="2:8" ht="21" x14ac:dyDescent="0.4">
       <c r="B46" s="92"/>
       <c r="C46" s="93"/>
       <c r="D46" s="93"/>
       <c r="E46" s="94"/>
-      <c r="F46" s="15" t="s">
+      <c r="F46" s="101" t="s">
         <v>22</v>
       </c>
-      <c r="G46" s="16"/>
-      <c r="H46" s="17"/>
+      <c r="G46" s="102"/>
+      <c r="H46" s="8"/>
     </row>
     <row r="47" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B47" s="92"/>
       <c r="C47" s="93"/>
       <c r="D47" s="93"/>
       <c r="E47" s="94"/>
-      <c r="F47" s="18" t="s">
+      <c r="F47" s="107" t="s">
         <v>23</v>
       </c>
-      <c r="G47" s="19"/>
-      <c r="H47" s="20"/>
+      <c r="G47" s="108"/>
+      <c r="H47" s="109"/>
     </row>
     <row r="48" spans="2:8" ht="21" x14ac:dyDescent="0.4">
       <c r="B48" s="92"/>
       <c r="C48" s="93"/>
       <c r="D48" s="93"/>
       <c r="E48" s="94"/>
-      <c r="F48" s="16" t="s">
+      <c r="F48" s="102" t="s">
         <v>24</v>
       </c>
-      <c r="G48" s="16"/>
-      <c r="H48" s="17"/>
+      <c r="G48" s="102"/>
+      <c r="H48" s="8"/>
     </row>
     <row r="49" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B49" s="102"/>
-      <c r="C49" s="95"/>
-      <c r="D49" s="95"/>
-      <c r="E49" s="96"/>
-      <c r="F49" s="102"/>
-      <c r="G49" s="95"/>
-      <c r="H49" s="96"/>
-    </row>
-    <row r="50" spans="2:8" ht="9.6" customHeight="1" x14ac:dyDescent="0.35"/>
+      <c r="B49" s="95"/>
+      <c r="C49" s="96"/>
+      <c r="D49" s="96"/>
+      <c r="E49" s="97"/>
+      <c r="F49" s="95"/>
+      <c r="G49" s="96"/>
+      <c r="H49" s="97"/>
+    </row>
+    <row r="50" spans="2:8" ht="9.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B50" s="112"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="19"/>
+    </row>
     <row r="51" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B51" s="85" t="s">
+      <c r="B51" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="C51" s="78"/>
-      <c r="D51" s="78"/>
-      <c r="E51" s="78"/>
-      <c r="F51" s="78"/>
-      <c r="G51" s="78"/>
-      <c r="H51" s="111"/>
+      <c r="C51" s="52"/>
+      <c r="D51" s="52"/>
+      <c r="E51" s="52"/>
+      <c r="F51" s="52"/>
+      <c r="G51" s="52"/>
+      <c r="H51" s="110"/>
     </row>
     <row r="52" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B52" s="108" t="s">
+      <c r="B52" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C52" s="109"/>
-      <c r="D52" s="109"/>
-      <c r="E52" s="109"/>
-      <c r="F52" s="109"/>
-      <c r="G52" s="109"/>
-      <c r="H52" s="110"/>
+      <c r="C52" s="38"/>
+      <c r="D52" s="38"/>
+      <c r="E52" s="38"/>
+      <c r="F52" s="38"/>
+      <c r="G52" s="38"/>
+      <c r="H52" s="39"/>
     </row>
     <row r="53" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B53" s="107"/>
-      <c r="C53" s="107"/>
-      <c r="D53" s="107"/>
-      <c r="E53" s="107"/>
-      <c r="F53" s="107"/>
-      <c r="G53" s="107"/>
-      <c r="H53" s="107"/>
+      <c r="B53" s="106"/>
+      <c r="C53" s="106"/>
+      <c r="D53" s="106"/>
+      <c r="E53" s="106"/>
+      <c r="F53" s="106"/>
+      <c r="G53" s="106"/>
+      <c r="H53" s="106"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B54" s="87"/>
-      <c r="C54" s="88"/>
-      <c r="D54" s="88"/>
-      <c r="E54" s="88"/>
-      <c r="F54" s="88"/>
-      <c r="G54" s="88"/>
-      <c r="H54" s="89"/>
+      <c r="B54" s="103"/>
+      <c r="C54" s="104"/>
+      <c r="D54" s="104"/>
+      <c r="E54" s="104"/>
+      <c r="F54" s="104"/>
+      <c r="G54" s="104"/>
+      <c r="H54" s="105"/>
     </row>
     <row r="55" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B55" s="85" t="s">
+      <c r="B55" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="C55" s="78"/>
-      <c r="D55" s="78"/>
-      <c r="E55" s="78"/>
-      <c r="F55" s="78"/>
-      <c r="G55" s="78"/>
-      <c r="H55" s="37"/>
+      <c r="C55" s="52"/>
+      <c r="D55" s="52"/>
+      <c r="E55" s="52"/>
+      <c r="F55" s="52"/>
+      <c r="G55" s="52"/>
+      <c r="H55" s="71"/>
     </row>
     <row r="56" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B56" s="85"/>
-      <c r="C56" s="78"/>
-      <c r="D56" s="78"/>
-      <c r="E56" s="78"/>
-      <c r="F56" s="78"/>
-      <c r="G56" s="78"/>
-      <c r="H56" s="37"/>
+      <c r="B56" s="51"/>
+      <c r="C56" s="52"/>
+      <c r="D56" s="52"/>
+      <c r="E56" s="52"/>
+      <c r="F56" s="52"/>
+      <c r="G56" s="52"/>
+      <c r="H56" s="71"/>
     </row>
     <row r="57" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B57" s="85" t="s">
+      <c r="B57" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="78"/>
-      <c r="F57" s="78"/>
-      <c r="G57" s="78"/>
-      <c r="H57" s="37"/>
+      <c r="C57" s="52"/>
+      <c r="D57" s="52"/>
+      <c r="E57" s="52"/>
+      <c r="F57" s="52"/>
+      <c r="G57" s="52"/>
+      <c r="H57" s="71"/>
     </row>
     <row r="58" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B58" s="85" t="s">
+      <c r="B58" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="C58" s="78"/>
-      <c r="D58" s="78"/>
-      <c r="E58" s="78"/>
-      <c r="F58" s="78"/>
-      <c r="G58" s="78"/>
-      <c r="H58" s="37"/>
+      <c r="C58" s="52"/>
+      <c r="D58" s="52"/>
+      <c r="E58" s="52"/>
+      <c r="F58" s="52"/>
+      <c r="G58" s="52"/>
+      <c r="H58" s="71"/>
     </row>
     <row r="59" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B59" s="85" t="s">
+      <c r="B59" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C59" s="78"/>
-      <c r="D59" s="78"/>
-      <c r="E59" s="78"/>
-      <c r="F59" s="78"/>
-      <c r="G59" s="78"/>
-      <c r="H59" s="37"/>
+      <c r="C59" s="52"/>
+      <c r="D59" s="52"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52"/>
+      <c r="G59" s="52"/>
+      <c r="H59" s="71"/>
     </row>
     <row r="60" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B60" s="104"/>
-      <c r="C60" s="90"/>
-      <c r="D60" s="90"/>
-      <c r="E60" s="90"/>
-      <c r="F60" s="90"/>
-      <c r="G60" s="90"/>
-      <c r="H60" s="91"/>
+      <c r="B60" s="77"/>
+      <c r="C60" s="78"/>
+      <c r="D60" s="78"/>
+      <c r="E60" s="78"/>
+      <c r="F60" s="78"/>
+      <c r="G60" s="78"/>
+      <c r="H60" s="79"/>
     </row>
     <row r="61" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B61" s="105" t="s">
+      <c r="B61" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="C61" s="106"/>
-      <c r="D61" s="80"/>
-      <c r="E61" s="80"/>
-      <c r="F61" s="81" t="s">
+      <c r="C61" s="74"/>
+      <c r="D61" s="75"/>
+      <c r="E61" s="75"/>
+      <c r="F61" s="76" t="s">
         <v>36</v>
       </c>
-      <c r="G61" s="81"/>
-      <c r="H61" s="81"/>
+      <c r="G61" s="76"/>
+      <c r="H61" s="76"/>
     </row>
     <row r="62" spans="2:8" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B62" s="105" t="s">
+      <c r="B62" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="C62" s="106"/>
-      <c r="D62" s="80"/>
-      <c r="E62" s="80"/>
-      <c r="F62" s="81" t="s">
+      <c r="C62" s="74"/>
+      <c r="D62" s="75"/>
+      <c r="E62" s="75"/>
+      <c r="F62" s="76" t="s">
         <v>37</v>
       </c>
-      <c r="G62" s="81"/>
-      <c r="H62" s="81"/>
+      <c r="G62" s="76"/>
+      <c r="H62" s="76"/>
     </row>
     <row r="63" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="105" t="s">
+      <c r="B63" s="73" t="s">
         <v>43</v>
       </c>
-      <c r="C63" s="106"/>
-      <c r="D63" s="80"/>
-      <c r="E63" s="80"/>
-      <c r="F63" s="81" t="s">
+      <c r="C63" s="74"/>
+      <c r="D63" s="75"/>
+      <c r="E63" s="75"/>
+      <c r="F63" s="76" t="s">
         <v>44</v>
       </c>
-      <c r="G63" s="81"/>
-      <c r="H63" s="81"/>
+      <c r="G63" s="76"/>
+      <c r="H63" s="76"/>
     </row>
     <row r="64" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
+      <c r="D64" s="72"/>
+      <c r="E64" s="72"/>
     </row>
     <row r="65" spans="4:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="D65" s="14"/>
-      <c r="E65" s="14"/>
+      <c r="D65" s="72"/>
+      <c r="E65" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="65">
@@ -2059,6 +2068,8 @@
     <mergeCell ref="B53:H53"/>
     <mergeCell ref="F47:H47"/>
     <mergeCell ref="C33:D33"/>
+    <mergeCell ref="B51:H51"/>
+    <mergeCell ref="C42:D42"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="C6:F9"/>
     <mergeCell ref="B46:E46"/>
@@ -2066,6 +2077,15 @@
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="F49:H49"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="B43:H43"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="F48:G48"/>
     <mergeCell ref="B56:H56"/>
     <mergeCell ref="B58:H58"/>
     <mergeCell ref="D64:E64"/>
@@ -2080,18 +2100,6 @@
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="B60:H60"/>
     <mergeCell ref="B57:H57"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="B43:H43"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="B51:H51"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="G21:H21"/>
     <mergeCell ref="B23:H23"/>
     <mergeCell ref="B25:G25"/>
     <mergeCell ref="C41:D41"/>
@@ -2106,7 +2114,6 @@
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C38:D38"/>
-    <mergeCell ref="F17:H17"/>
     <mergeCell ref="G19:H19"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B11:C11"/>
@@ -2115,10 +2122,12 @@
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B15:C15"/>
+    <mergeCell ref="G21:H21"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G9:H9"/>
+    <mergeCell ref="F17:H17"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="52" orientation="portrait" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Arreglo de FIRMAS EN FORMATOS
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO ODC.xlsx
+++ b/storage/app/templates/FORMATO ODC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adv\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E21DC67-161A-4D6C-A076-BA66186F845E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42D2AAE-B275-41B5-9D61-41880E721285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="1" xr2:uid="{CD2C727A-B478-40DC-A0A5-37EBD1630B47}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="REFERENICA ODC" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'REFERENICA ODC'!$B$6:$H$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'REFERENICA ODC'!$B$6:$H$65</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="52">
   <si>
     <t>TOTAL</t>
   </si>
@@ -274,12 +274,6 @@
     <t>{{cantidad}}</t>
   </si>
   <si>
-    <t>FIRMA: {{firma_elaborado}}</t>
-  </si>
-  <si>
-    <t>FIRMA: {{firma_aprobado}}</t>
-  </si>
-  <si>
     <t>{{empresa_direccion_fiscal}}</t>
   </si>
   <si>
@@ -293,6 +287,18 @@
   </si>
   <si>
     <t>PROVEEDOR: {{proveedor_nombre}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIRMA: </t>
+  </si>
+  <si>
+    <t>{{firma_elaborado}}</t>
+  </si>
+  <si>
+    <t>{{firma_aprobado}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                  </t>
   </si>
 </sst>
 </file>
@@ -603,7 +609,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -697,16 +703,170 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -727,12 +887,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -751,166 +905,39 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares 3" xfId="2" xr:uid="{60AA6EFA-E802-43AC-A264-3B3C3439C925}"/>
@@ -1306,7 +1333,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B6:H65"/>
+  <dimension ref="B6:H66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="26" defaultRowHeight="20.399999999999999" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" style="1"/>
@@ -1316,50 +1343,50 @@
   </cols>
   <sheetData>
     <row r="6" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="80"/>
-      <c r="C6" s="83" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="84"/>
-      <c r="E6" s="84"/>
-      <c r="F6" s="85"/>
-      <c r="G6" s="41" t="s">
+      <c r="B6" s="55"/>
+      <c r="C6" s="58" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="42"/>
+      <c r="H6" s="110"/>
     </row>
     <row r="7" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="81"/>
-      <c r="C7" s="86"/>
-      <c r="D7" s="87"/>
-      <c r="E7" s="87"/>
-      <c r="F7" s="88"/>
-      <c r="G7" s="41" t="s">
+      <c r="B7" s="56"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="42"/>
+      <c r="H7" s="110"/>
     </row>
     <row r="8" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="81"/>
-      <c r="C8" s="86"/>
-      <c r="D8" s="87"/>
-      <c r="E8" s="87"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="41" t="s">
+      <c r="B8" s="56"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="63"/>
+      <c r="G8" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="42"/>
+      <c r="H8" s="110"/>
     </row>
     <row r="9" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="82"/>
-      <c r="C9" s="89"/>
-      <c r="D9" s="90"/>
-      <c r="E9" s="90"/>
-      <c r="F9" s="91"/>
-      <c r="G9" s="41" t="s">
+      <c r="B9" s="57"/>
+      <c r="C9" s="64"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="109" t="s">
         <v>7</v>
       </c>
-      <c r="H9" s="42"/>
+      <c r="H9" s="110"/>
     </row>
     <row r="10" spans="2:8" ht="21" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
@@ -1371,10 +1398,10 @@
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="2:8" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="49" t="s">
+      <c r="B11" s="101" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="50"/>
+      <c r="C11" s="102"/>
       <c r="D11" s="16"/>
       <c r="E11" s="17"/>
       <c r="F11" s="17"/>
@@ -1382,36 +1409,36 @@
       <c r="H11" s="19"/>
     </row>
     <row r="12" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="51" t="s">
+      <c r="B12" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="52"/>
+      <c r="C12" s="44"/>
       <c r="D12" s="20"/>
       <c r="E12" s="21"/>
       <c r="F12" s="22"/>
-      <c r="G12" s="53" t="s">
+      <c r="G12" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="54"/>
+      <c r="H12" s="104"/>
     </row>
     <row r="13" spans="2:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B13" s="32" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="20"/>
       <c r="E13" s="21"/>
       <c r="F13" s="21"/>
-      <c r="G13" s="53" t="s">
+      <c r="G13" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="H13" s="54"/>
+      <c r="H13" s="104"/>
     </row>
     <row r="14" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="51" t="s">
+      <c r="B14" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="52"/>
+      <c r="C14" s="44"/>
       <c r="D14" s="27"/>
       <c r="E14" s="21"/>
       <c r="F14" s="21"/>
@@ -1419,8 +1446,8 @@
       <c r="H14" s="28"/>
     </row>
     <row r="15" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B15" s="55"/>
-      <c r="C15" s="56"/>
+      <c r="B15" s="105"/>
+      <c r="C15" s="106"/>
       <c r="D15" s="29"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
@@ -1432,14 +1459,14 @@
     </row>
     <row r="17" spans="2:8" ht="39" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="33" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="44"/>
+      <c r="F17" s="111"/>
+      <c r="G17" s="111"/>
+      <c r="H17" s="112"/>
     </row>
     <row r="18" spans="2:8" ht="6.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="36"/>
@@ -1458,10 +1485,10 @@
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
-      <c r="G19" s="45" t="s">
+      <c r="G19" s="97" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="46"/>
+      <c r="H19" s="98"/>
     </row>
     <row r="20" spans="2:8" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="36"/>
@@ -1473,17 +1500,17 @@
       <c r="H20" s="11"/>
     </row>
     <row r="21" spans="2:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="47" t="s">
+      <c r="B21" s="99" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="57" t="s">
+      <c r="C21" s="100"/>
+      <c r="D21" s="100"/>
+      <c r="E21" s="100"/>
+      <c r="F21" s="100"/>
+      <c r="G21" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="58"/>
+      <c r="H21" s="108"/>
     </row>
     <row r="22" spans="2:8" ht="12.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="12"/>
@@ -1495,15 +1522,15 @@
       <c r="H22" s="13"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="60"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="61"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="87"/>
+      <c r="E23" s="87"/>
+      <c r="F23" s="87"/>
+      <c r="G23" s="87"/>
+      <c r="H23" s="88"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B24" s="12"/>
@@ -1515,14 +1542,14 @@
       <c r="H24" s="13"/>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B25" s="59" t="s">
+      <c r="B25" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="60"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="60"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="87"/>
+      <c r="F25" s="87"/>
+      <c r="G25" s="87"/>
       <c r="H25" s="13"/>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.35">
@@ -1535,15 +1562,15 @@
       <c r="H26" s="13"/>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B27" s="68" t="s">
+      <c r="B27" s="94" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="69"/>
-      <c r="D27" s="69"/>
-      <c r="E27" s="69"/>
-      <c r="F27" s="69"/>
-      <c r="G27" s="69"/>
-      <c r="H27" s="70"/>
+      <c r="C27" s="95"/>
+      <c r="D27" s="95"/>
+      <c r="E27" s="95"/>
+      <c r="F27" s="95"/>
+      <c r="G27" s="95"/>
+      <c r="H27" s="96"/>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B28" s="5"/>
@@ -1564,17 +1591,17 @@
       <c r="H29" s="31"/>
     </row>
     <row r="30" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B30" s="63" t="s">
+      <c r="B30" s="89" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="65" t="s">
+      <c r="C30" s="91" t="s">
         <v>5</v>
       </c>
-      <c r="D30" s="66"/>
-      <c r="E30" s="67" t="s">
+      <c r="D30" s="92"/>
+      <c r="E30" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="F30" s="67" t="s">
+      <c r="F30" s="93" t="s">
         <v>3</v>
       </c>
       <c r="G30" s="4" t="s">
@@ -1585,11 +1612,11 @@
       </c>
     </row>
     <row r="31" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B31" s="64"/>
-      <c r="C31" s="65"/>
-      <c r="D31" s="66"/>
-      <c r="E31" s="67"/>
-      <c r="F31" s="67"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="91"/>
+      <c r="D31" s="92"/>
+      <c r="E31" s="93"/>
+      <c r="F31" s="93"/>
       <c r="G31" s="4" t="s">
         <v>1</v>
       </c>
@@ -1601,310 +1628,310 @@
       <c r="B32" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="62" t="s">
+      <c r="C32" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="62"/>
+      <c r="D32" s="53"/>
       <c r="E32" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F32" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G32" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H32" s="111" t="s">
-        <v>47</v>
+      <c r="G32" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H32" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:8" ht="19.8" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C33" s="62" t="s">
+      <c r="C33" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D33" s="62"/>
+      <c r="D33" s="53"/>
       <c r="E33" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F33" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G33" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H33" s="111" t="s">
-        <v>47</v>
+      <c r="G33" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H33" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="62" t="s">
+      <c r="C34" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D34" s="62"/>
+      <c r="D34" s="53"/>
       <c r="E34" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F34" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G34" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H34" s="111" t="s">
-        <v>47</v>
+      <c r="G34" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H34" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="2:8" ht="16.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="62" t="s">
+      <c r="C35" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D35" s="62"/>
+      <c r="D35" s="53"/>
       <c r="E35" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F35" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G35" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H35" s="111" t="s">
-        <v>47</v>
+      <c r="G35" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H35" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B36" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="62" t="s">
+      <c r="C36" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="62"/>
+      <c r="D36" s="53"/>
       <c r="E36" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F36" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G36" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H36" s="111" t="s">
-        <v>47</v>
+      <c r="G36" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H36" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B37" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C37" s="62" t="s">
+      <c r="C37" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D37" s="62"/>
+      <c r="D37" s="53"/>
       <c r="E37" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F37" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G37" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H37" s="111" t="s">
-        <v>47</v>
+      <c r="G37" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H37" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B38" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="62" t="s">
+      <c r="C38" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D38" s="62"/>
+      <c r="D38" s="53"/>
       <c r="E38" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F38" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G38" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H38" s="111" t="s">
-        <v>47</v>
+      <c r="G38" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H38" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B39" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="62" t="s">
+      <c r="C39" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D39" s="62"/>
+      <c r="D39" s="53"/>
       <c r="E39" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F39" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G39" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H39" s="111" t="s">
-        <v>47</v>
+      <c r="G39" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H39" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B40" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C40" s="62" t="s">
+      <c r="C40" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D40" s="62"/>
+      <c r="D40" s="53"/>
       <c r="E40" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F40" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G40" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H40" s="111" t="s">
-        <v>47</v>
+      <c r="G40" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H40" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B41" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C41" s="62" t="s">
+      <c r="C41" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D41" s="62"/>
+      <c r="D41" s="53"/>
       <c r="E41" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F41" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G41" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H41" s="111" t="s">
-        <v>47</v>
+      <c r="G41" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H41" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B42" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="C42" s="62" t="s">
+      <c r="C42" s="53" t="s">
         <v>40</v>
       </c>
-      <c r="D42" s="62"/>
+      <c r="D42" s="53"/>
       <c r="E42" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F42" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="G42" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="H42" s="111" t="s">
-        <v>47</v>
+      <c r="G42" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H42" s="41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B43" s="98"/>
-      <c r="C43" s="98"/>
-      <c r="D43" s="98"/>
-      <c r="E43" s="98"/>
-      <c r="F43" s="98"/>
-      <c r="G43" s="98"/>
-      <c r="H43" s="98"/>
+      <c r="B43" s="73"/>
+      <c r="C43" s="73"/>
+      <c r="D43" s="73"/>
+      <c r="E43" s="73"/>
+      <c r="F43" s="73"/>
+      <c r="G43" s="73"/>
+      <c r="H43" s="73"/>
     </row>
     <row r="44" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B44" s="99"/>
-      <c r="C44" s="100"/>
-      <c r="D44" s="100"/>
-      <c r="E44" s="100"/>
-      <c r="F44" s="101" t="s">
+      <c r="B44" s="74"/>
+      <c r="C44" s="75"/>
+      <c r="D44" s="75"/>
+      <c r="E44" s="75"/>
+      <c r="F44" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="G44" s="102"/>
+      <c r="G44" s="77"/>
       <c r="H44" s="8"/>
     </row>
     <row r="45" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B45" s="101" t="s">
+      <c r="B45" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="C45" s="102"/>
-      <c r="D45" s="102"/>
-      <c r="E45" s="102"/>
-      <c r="F45" s="101" t="s">
+      <c r="C45" s="77"/>
+      <c r="D45" s="77"/>
+      <c r="E45" s="77"/>
+      <c r="F45" s="76" t="s">
         <v>21</v>
       </c>
-      <c r="G45" s="102"/>
+      <c r="G45" s="77"/>
       <c r="H45" s="8"/>
     </row>
     <row r="46" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B46" s="92"/>
-      <c r="C46" s="93"/>
-      <c r="D46" s="93"/>
-      <c r="E46" s="94"/>
-      <c r="F46" s="101" t="s">
+      <c r="B46" s="67"/>
+      <c r="C46" s="68"/>
+      <c r="D46" s="68"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="G46" s="102"/>
+      <c r="G46" s="77"/>
       <c r="H46" s="8"/>
     </row>
     <row r="47" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="92"/>
-      <c r="C47" s="93"/>
-      <c r="D47" s="93"/>
-      <c r="E47" s="94"/>
-      <c r="F47" s="107" t="s">
+      <c r="B47" s="67"/>
+      <c r="C47" s="68"/>
+      <c r="D47" s="68"/>
+      <c r="E47" s="69"/>
+      <c r="F47" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="G47" s="108"/>
-      <c r="H47" s="109"/>
+      <c r="G47" s="51"/>
+      <c r="H47" s="52"/>
     </row>
     <row r="48" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B48" s="92"/>
-      <c r="C48" s="93"/>
-      <c r="D48" s="93"/>
-      <c r="E48" s="94"/>
-      <c r="F48" s="102" t="s">
+      <c r="B48" s="67"/>
+      <c r="C48" s="68"/>
+      <c r="D48" s="68"/>
+      <c r="E48" s="69"/>
+      <c r="F48" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G48" s="102"/>
+      <c r="G48" s="77"/>
       <c r="H48" s="8"/>
     </row>
     <row r="49" spans="2:8" ht="21" x14ac:dyDescent="0.4">
-      <c r="B49" s="95"/>
-      <c r="C49" s="96"/>
-      <c r="D49" s="96"/>
-      <c r="E49" s="97"/>
-      <c r="F49" s="95"/>
-      <c r="G49" s="96"/>
-      <c r="H49" s="97"/>
+      <c r="B49" s="70"/>
+      <c r="C49" s="71"/>
+      <c r="D49" s="71"/>
+      <c r="E49" s="72"/>
+      <c r="F49" s="70"/>
+      <c r="G49" s="71"/>
+      <c r="H49" s="72"/>
     </row>
     <row r="50" spans="2:8" ht="9.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="112"/>
+      <c r="B50" s="42"/>
       <c r="C50" s="18"/>
       <c r="D50" s="18"/>
       <c r="E50" s="18"/>
@@ -1913,15 +1940,15 @@
       <c r="H50" s="19"/>
     </row>
     <row r="51" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B51" s="51" t="s">
+      <c r="B51" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="C51" s="52"/>
-      <c r="D51" s="52"/>
-      <c r="E51" s="52"/>
-      <c r="F51" s="52"/>
-      <c r="G51" s="52"/>
-      <c r="H51" s="110"/>
+      <c r="C51" s="44"/>
+      <c r="D51" s="44"/>
+      <c r="E51" s="44"/>
+      <c r="F51" s="44"/>
+      <c r="G51" s="44"/>
+      <c r="H51" s="54"/>
     </row>
     <row r="52" spans="2:8" ht="21" x14ac:dyDescent="0.4">
       <c r="B52" s="37" t="s">
@@ -1935,141 +1962,191 @@
       <c r="H52" s="39"/>
     </row>
     <row r="53" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B53" s="106"/>
-      <c r="C53" s="106"/>
-      <c r="D53" s="106"/>
-      <c r="E53" s="106"/>
-      <c r="F53" s="106"/>
-      <c r="G53" s="106"/>
-      <c r="H53" s="106"/>
+      <c r="B53" s="49"/>
+      <c r="C53" s="49"/>
+      <c r="D53" s="49"/>
+      <c r="E53" s="49"/>
+      <c r="F53" s="49"/>
+      <c r="G53" s="49"/>
+      <c r="H53" s="49"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B54" s="103"/>
-      <c r="C54" s="104"/>
-      <c r="D54" s="104"/>
-      <c r="E54" s="104"/>
-      <c r="F54" s="104"/>
-      <c r="G54" s="104"/>
-      <c r="H54" s="105"/>
+      <c r="B54" s="46"/>
+      <c r="C54" s="47"/>
+      <c r="D54" s="47"/>
+      <c r="E54" s="47"/>
+      <c r="F54" s="47"/>
+      <c r="G54" s="47"/>
+      <c r="H54" s="48"/>
     </row>
     <row r="55" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B55" s="51" t="s">
+      <c r="B55" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="C55" s="52"/>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="52"/>
-      <c r="H55" s="71"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="44"/>
+      <c r="F55" s="44"/>
+      <c r="G55" s="44"/>
+      <c r="H55" s="45"/>
     </row>
     <row r="56" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B56" s="51"/>
-      <c r="C56" s="52"/>
-      <c r="D56" s="52"/>
-      <c r="E56" s="52"/>
-      <c r="F56" s="52"/>
-      <c r="G56" s="52"/>
-      <c r="H56" s="71"/>
+      <c r="B56" s="43"/>
+      <c r="C56" s="44"/>
+      <c r="D56" s="44"/>
+      <c r="E56" s="44"/>
+      <c r="F56" s="44"/>
+      <c r="G56" s="44"/>
+      <c r="H56" s="45"/>
     </row>
     <row r="57" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B57" s="51" t="s">
+      <c r="B57" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="C57" s="52"/>
-      <c r="D57" s="52"/>
-      <c r="E57" s="52"/>
-      <c r="F57" s="52"/>
-      <c r="G57" s="52"/>
-      <c r="H57" s="71"/>
+      <c r="C57" s="44"/>
+      <c r="D57" s="44"/>
+      <c r="E57" s="44"/>
+      <c r="F57" s="44"/>
+      <c r="G57" s="44"/>
+      <c r="H57" s="45"/>
     </row>
     <row r="58" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B58" s="51" t="s">
+      <c r="B58" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="C58" s="52"/>
-      <c r="D58" s="52"/>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="52"/>
-      <c r="H58" s="71"/>
+      <c r="C58" s="44"/>
+      <c r="D58" s="44"/>
+      <c r="E58" s="44"/>
+      <c r="F58" s="44"/>
+      <c r="G58" s="44"/>
+      <c r="H58" s="45"/>
     </row>
     <row r="59" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B59" s="51" t="s">
+      <c r="B59" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="71"/>
+      <c r="C59" s="44"/>
+      <c r="D59" s="44"/>
+      <c r="E59" s="44"/>
+      <c r="F59" s="44"/>
+      <c r="G59" s="44"/>
+      <c r="H59" s="45"/>
     </row>
     <row r="60" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="B60" s="77"/>
-      <c r="C60" s="78"/>
-      <c r="D60" s="78"/>
-      <c r="E60" s="78"/>
-      <c r="F60" s="78"/>
-      <c r="G60" s="78"/>
-      <c r="H60" s="79"/>
+      <c r="B60" s="83"/>
+      <c r="C60" s="84"/>
+      <c r="D60" s="84"/>
+      <c r="E60" s="84"/>
+      <c r="F60" s="84"/>
+      <c r="G60" s="84"/>
+      <c r="H60" s="85"/>
     </row>
     <row r="61" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B61" s="73" t="s">
+      <c r="B61" s="79" t="s">
         <v>35</v>
       </c>
-      <c r="C61" s="74"/>
-      <c r="D61" s="75"/>
-      <c r="E61" s="75"/>
-      <c r="F61" s="76" t="s">
+      <c r="C61" s="80"/>
+      <c r="D61" s="81"/>
+      <c r="E61" s="81"/>
+      <c r="F61" s="82" t="s">
         <v>36</v>
       </c>
-      <c r="G61" s="76"/>
-      <c r="H61" s="76"/>
+      <c r="G61" s="82"/>
+      <c r="H61" s="82"/>
     </row>
     <row r="62" spans="2:8" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B62" s="73" t="s">
+      <c r="B62" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="C62" s="74"/>
-      <c r="D62" s="75"/>
-      <c r="E62" s="75"/>
-      <c r="F62" s="76" t="s">
+      <c r="C62" s="80"/>
+      <c r="D62" s="81"/>
+      <c r="E62" s="81"/>
+      <c r="F62" s="82" t="s">
         <v>37</v>
       </c>
-      <c r="G62" s="76"/>
-      <c r="H62" s="76"/>
-    </row>
-    <row r="63" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B63" s="73" t="s">
-        <v>43</v>
-      </c>
-      <c r="C63" s="74"/>
-      <c r="D63" s="75"/>
-      <c r="E63" s="75"/>
-      <c r="F63" s="76" t="s">
-        <v>44</v>
-      </c>
-      <c r="G63" s="76"/>
-      <c r="H63" s="76"/>
-    </row>
-    <row r="64" spans="2:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="D64" s="72"/>
-      <c r="E64" s="72"/>
+      <c r="G62" s="82"/>
+      <c r="H62" s="82"/>
+    </row>
+    <row r="63" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B63" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="C63" s="118"/>
+      <c r="D63" s="81"/>
+      <c r="E63" s="81"/>
+      <c r="F63" s="117" t="s">
+        <v>51</v>
+      </c>
+      <c r="G63" s="119" t="s">
+        <v>50</v>
+      </c>
+      <c r="H63" s="116"/>
+    </row>
+    <row r="64" spans="2:8" ht="51.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B64" s="113" t="s">
+        <v>48</v>
+      </c>
+      <c r="C64" s="114"/>
+      <c r="D64" s="81"/>
+      <c r="E64" s="81"/>
+      <c r="F64" s="115" t="s">
+        <v>48</v>
+      </c>
+      <c r="G64" s="115"/>
+      <c r="H64" s="115"/>
     </row>
     <row r="65" spans="4:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="D65" s="72"/>
-      <c r="E65" s="72"/>
+      <c r="D65" s="78"/>
+      <c r="E65" s="78"/>
+    </row>
+    <row r="66" spans="4:5" ht="21" x14ac:dyDescent="0.35">
+      <c r="D66" s="78"/>
+      <c r="E66" s="78"/>
     </row>
   </sheetData>
   <mergeCells count="65">
-    <mergeCell ref="B55:H55"/>
-    <mergeCell ref="B54:H54"/>
-    <mergeCell ref="B53:H53"/>
-    <mergeCell ref="F47:H47"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="B51:H51"/>
-    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="B56:H56"/>
+    <mergeCell ref="B58:H58"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="D61:E64"/>
+    <mergeCell ref="F61:H61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="F62:H62"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="F64:H64"/>
+    <mergeCell ref="B59:H59"/>
+    <mergeCell ref="B60:H60"/>
+    <mergeCell ref="B57:H57"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="C6:F9"/>
     <mergeCell ref="B46:E46"/>
@@ -2086,51 +2163,16 @@
     <mergeCell ref="F45:G45"/>
     <mergeCell ref="F46:G46"/>
     <mergeCell ref="F48:G48"/>
-    <mergeCell ref="B56:H56"/>
-    <mergeCell ref="B58:H58"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="D61:E63"/>
-    <mergeCell ref="F61:H61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="F62:H62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="F63:H63"/>
-    <mergeCell ref="B59:H59"/>
-    <mergeCell ref="B60:H60"/>
-    <mergeCell ref="B57:H57"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="B27:H27"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="B55:H55"/>
+    <mergeCell ref="B54:H54"/>
+    <mergeCell ref="B53:H53"/>
+    <mergeCell ref="F47:H47"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="B51:H51"/>
+    <mergeCell ref="C42:D42"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="52" orientation="portrait" verticalDpi="300" r:id="rId1"/>
+  <pageSetup scale="49" orientation="portrait" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>